<commit_message>
Feat: increased PTC current rating, dropped R5 to ensure saturation on Q2
Also switched all parts (except the battery case) to a KiCad library part to update. Moving the design to KiCad (r.i.p Eagle).

Increased current rating of PTC1 to 2.5A hold, 5A trip to reduce possibility of inadvertent tripping.
Dropped R5 to ensure saturation on Q2
Q2 is surprisingly able to handle the pulse current. Peak pulse is 6A, which should cover requirement. Maybe consider ZTX618 instead, which has a higher amp rating.
Q2 (ZTX718) is being retired, so if you're reading this you need to pick a different part.
</commit_message>
<xml_diff>
--- a/LaunchController1 BOM.xlsx
+++ b/LaunchController1 BOM.xlsx
@@ -1,18 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\MR-Launch-Controller\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{588297AE-1491-496B-B4A3-ED6F528889F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="My Lists Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="100">
   <si>
     <t>Index</t>
   </si>
@@ -269,24 +277,9 @@
     <t>D1, D2</t>
   </si>
   <si>
-    <t>0ZRG0120FF2E</t>
-  </si>
-  <si>
     <t>Bel Fuse Inc.</t>
   </si>
   <si>
-    <t>PTC RESET FUSE 30V 1.2A RADIAL</t>
-  </si>
-  <si>
-    <t>507-0ZRG0120FF2ECT-ND</t>
-  </si>
-  <si>
-    <t>0.44000</t>
-  </si>
-  <si>
-    <t>$0.44</t>
-  </si>
-  <si>
     <t>PTC1</t>
   </si>
   <si>
@@ -318,14 +311,22 @@
   </si>
   <si>
     <t>R2, R3, R6</t>
+  </si>
+  <si>
+    <t>0ZRG0250FF1E</t>
+  </si>
+  <si>
+    <t>PTC RESET FUSE 30V 2.5A RADIAL</t>
+  </si>
+  <si>
+    <t>5923-0ZRG0250FF1E-ND</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -349,677 +350,985 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="4" max="4" width="29.21875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="0" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="0" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="0" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="0">
-        <v>1</v>
-      </c>
-      <c r="G2" s="0">
-        <v>1</v>
-      </c>
-      <c r="H2" s="0" t="s">
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="J2" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="0">
-        <v>1</v>
-      </c>
-      <c r="M2" s="0" t="s">
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
         <v>24</v>
       </c>
-      <c r="N2" s="0" t="s">
+      <c r="N2" t="s">
         <v>25</v>
       </c>
-      <c r="O2" s="0" t="s">
+      <c r="O2" t="s">
         <v>26</v>
       </c>
-      <c r="P2" s="0" t="s">
+      <c r="P2" t="s">
         <v>27</v>
       </c>
-      <c r="Q2" s="0" t="s">
+      <c r="Q2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="0">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="0">
-        <v>1</v>
-      </c>
-      <c r="G3" s="0">
-        <v>1</v>
-      </c>
-      <c r="H3" s="0" t="s">
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="J3" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="K3" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="0">
-        <v>1</v>
-      </c>
-      <c r="M3" s="0" t="s">
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
         <v>35</v>
       </c>
-      <c r="N3" s="0" t="s">
+      <c r="N3" t="s">
         <v>25</v>
       </c>
-      <c r="O3" s="0" t="s">
+      <c r="O3" t="s">
         <v>26</v>
       </c>
-      <c r="P3" s="0" t="s">
+      <c r="P3" t="s">
         <v>27</v>
       </c>
-      <c r="Q3" s="0" t="s">
+      <c r="Q3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="0">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" t="s">
         <v>37</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="0">
+      <c r="F4">
         <v>2</v>
       </c>
-      <c r="G4" s="0">
+      <c r="G4">
         <v>2</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="H4" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="I4" t="s">
         <v>40</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="J4" t="s">
         <v>41</v>
       </c>
-      <c r="K4" s="0" t="s">
+      <c r="K4" t="s">
         <v>34</v>
       </c>
-      <c r="L4" s="0">
-        <v>1</v>
-      </c>
-      <c r="M4" s="0" t="s">
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
         <v>25</v>
       </c>
-      <c r="N4" s="0" t="s">
+      <c r="N4" t="s">
         <v>25</v>
       </c>
-      <c r="O4" s="0" t="s">
+      <c r="O4" t="s">
         <v>26</v>
       </c>
-      <c r="P4" s="0" t="s">
+      <c r="P4" t="s">
         <v>42</v>
       </c>
-      <c r="Q4" s="0" t="s">
+      <c r="Q4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="0">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" t="s">
         <v>45</v>
       </c>
-      <c r="F5" s="0">
-        <v>1</v>
-      </c>
-      <c r="G5" s="0">
-        <v>1</v>
-      </c>
-      <c r="H5" s="0" t="s">
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="I5" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="0" t="s">
+      <c r="J5" t="s">
         <v>47</v>
       </c>
-      <c r="K5" s="0" t="s">
+      <c r="K5" t="s">
         <v>48</v>
       </c>
-      <c r="L5" s="0">
-        <v>1</v>
-      </c>
-      <c r="M5" s="0" t="s">
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
         <v>49</v>
       </c>
-      <c r="N5" s="0" t="s">
+      <c r="N5" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="0" t="s">
+      <c r="O5" t="s">
         <v>26</v>
       </c>
-      <c r="P5" s="0" t="s">
+      <c r="P5" t="s">
         <v>42</v>
       </c>
-      <c r="Q5" s="0" t="s">
+      <c r="Q5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="0">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="0">
-        <v>1</v>
-      </c>
-      <c r="G6" s="0">
-        <v>1</v>
-      </c>
-      <c r="H6" s="0" t="s">
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
         <v>52</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="I6" t="s">
         <v>53</v>
       </c>
-      <c r="J6" s="0" t="s">
+      <c r="J6" t="s">
         <v>54</v>
       </c>
-      <c r="K6" s="0" t="s">
+      <c r="K6" t="s">
         <v>55</v>
       </c>
-      <c r="L6" s="0">
-        <v>1</v>
-      </c>
-      <c r="M6" s="0" t="s">
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
         <v>56</v>
       </c>
-      <c r="N6" s="0" t="s">
+      <c r="N6" t="s">
         <v>25</v>
       </c>
-      <c r="O6" s="0" t="s">
+      <c r="O6" t="s">
         <v>26</v>
       </c>
-      <c r="P6" s="0" t="s">
+      <c r="P6" t="s">
         <v>42</v>
       </c>
-      <c r="Q6" s="0" t="s">
+      <c r="Q6" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="0">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" t="s">
         <v>59</v>
       </c>
-      <c r="F7" s="0">
-        <v>1</v>
-      </c>
-      <c r="G7" s="0">
-        <v>1</v>
-      </c>
-      <c r="H7" s="0" t="s">
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="I7" t="s">
         <v>60</v>
       </c>
-      <c r="J7" s="0" t="s">
+      <c r="J7" t="s">
         <v>61</v>
       </c>
-      <c r="K7" s="0" t="s">
+      <c r="K7" t="s">
         <v>62</v>
       </c>
-      <c r="L7" s="0">
-        <v>1</v>
-      </c>
-      <c r="M7" s="0" t="s">
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
         <v>63</v>
       </c>
-      <c r="N7" s="0" t="s">
+      <c r="N7" t="s">
         <v>25</v>
       </c>
-      <c r="O7" s="0" t="s">
+      <c r="O7" t="s">
         <v>26</v>
       </c>
-      <c r="P7" s="0" t="s">
+      <c r="P7" t="s">
         <v>27</v>
       </c>
-      <c r="Q7" s="0" t="s">
+      <c r="Q7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="0">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" t="s">
         <v>65</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" t="s">
         <v>66</v>
       </c>
-      <c r="F8" s="0">
+      <c r="F8">
         <v>2</v>
       </c>
-      <c r="G8" s="0">
+      <c r="G8">
         <v>2</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="H8" t="s">
         <v>39</v>
       </c>
-      <c r="I8" s="0" t="s">
+      <c r="I8" t="s">
         <v>67</v>
       </c>
-      <c r="J8" s="0" t="s">
+      <c r="J8" t="s">
         <v>68</v>
       </c>
-      <c r="K8" s="0" t="s">
+      <c r="K8" t="s">
         <v>69</v>
       </c>
-      <c r="L8" s="0">
-        <v>1</v>
-      </c>
-      <c r="M8" s="0" t="s">
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
         <v>70</v>
       </c>
-      <c r="N8" s="0" t="s">
+      <c r="N8" t="s">
         <v>25</v>
       </c>
-      <c r="O8" s="0" t="s">
+      <c r="O8" t="s">
         <v>26</v>
       </c>
-      <c r="P8" s="0" t="s">
+      <c r="P8" t="s">
         <v>27</v>
       </c>
-      <c r="Q8" s="0" t="s">
+      <c r="Q8" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="0">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>71</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" t="s">
         <v>72</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" t="s">
         <v>73</v>
       </c>
-      <c r="F9" s="0">
-        <v>1</v>
-      </c>
-      <c r="G9" s="0">
-        <v>1</v>
-      </c>
-      <c r="H9" s="0" t="s">
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
         <v>39</v>
       </c>
-      <c r="I9" s="0" t="s">
+      <c r="I9" t="s">
         <v>74</v>
       </c>
-      <c r="J9" s="0" t="s">
+      <c r="J9" t="s">
         <v>75</v>
       </c>
-      <c r="K9" s="0" t="s">
+      <c r="K9" t="s">
         <v>76</v>
       </c>
-      <c r="L9" s="0">
-        <v>1</v>
-      </c>
-      <c r="M9" s="0" t="s">
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
         <v>77</v>
       </c>
-      <c r="N9" s="0" t="s">
+      <c r="N9" t="s">
         <v>25</v>
       </c>
-      <c r="O9" s="0" t="s">
+      <c r="O9" t="s">
         <v>26</v>
       </c>
-      <c r="P9" s="0" t="s">
+      <c r="P9" t="s">
         <v>42</v>
       </c>
-      <c r="Q9" s="0" t="s">
+      <c r="Q9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="0">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>78</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" t="s">
         <v>79</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" t="s">
         <v>80</v>
       </c>
-      <c r="F10" s="0">
+      <c r="F10">
         <v>2</v>
       </c>
-      <c r="G10" s="0">
+      <c r="G10">
         <v>2</v>
       </c>
-      <c r="H10" s="0" t="s">
+      <c r="H10" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="0" t="s">
+      <c r="I10" t="s">
         <v>81</v>
       </c>
-      <c r="J10" s="0" t="s">
+      <c r="J10" t="s">
         <v>82</v>
       </c>
-      <c r="K10" s="0" t="s">
+      <c r="K10" t="s">
         <v>83</v>
       </c>
-      <c r="L10" s="0">
-        <v>1</v>
-      </c>
-      <c r="M10" s="0" t="s">
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
         <v>84</v>
       </c>
-      <c r="N10" s="0" t="s">
+      <c r="N10" t="s">
         <v>25</v>
       </c>
-      <c r="O10" s="0" t="s">
+      <c r="O10" t="s">
         <v>26</v>
       </c>
-      <c r="P10" s="0" t="s">
+      <c r="P10" t="s">
         <v>27</v>
       </c>
-      <c r="Q10" s="0" t="s">
+      <c r="Q10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="0">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" t="s">
         <v>85</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="D11" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11" t="s">
+        <v>52</v>
+      </c>
+      <c r="I11" t="s">
+        <v>99</v>
+      </c>
+      <c r="J11">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="K11">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
         <v>86</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="N11" t="s">
+        <v>25</v>
+      </c>
+      <c r="O11" t="s">
+        <v>26</v>
+      </c>
+      <c r="P11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>87</v>
       </c>
-      <c r="F11" s="0">
-        <v>1</v>
-      </c>
-      <c r="G11" s="0">
-        <v>1</v>
-      </c>
-      <c r="H11" s="0" t="s">
+      <c r="C12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D12" t="s">
+        <v>89</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12">
+        <v>3</v>
+      </c>
+      <c r="H12" t="s">
         <v>52</v>
       </c>
-      <c r="I11" s="0" t="s">
+      <c r="I12" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" t="s">
+        <v>91</v>
+      </c>
+      <c r="K12" t="s">
+        <v>55</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>92</v>
+      </c>
+      <c r="N12" t="s">
+        <v>25</v>
+      </c>
+      <c r="O12" t="s">
+        <v>26</v>
+      </c>
+      <c r="P12" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" t="s">
         <v>88</v>
       </c>
-      <c r="J11" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="K11" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="L11" s="0">
-        <v>1</v>
-      </c>
-      <c r="M11" s="0" t="s">
+      <c r="D13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>3</v>
+      </c>
+      <c r="H13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I13" t="s">
+        <v>95</v>
+      </c>
+      <c r="J13" t="s">
         <v>91</v>
       </c>
-      <c r="N11" s="0" t="s">
+      <c r="K13" t="s">
+        <v>55</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>96</v>
+      </c>
+      <c r="N13" t="s">
         <v>25</v>
       </c>
-      <c r="O11" s="0" t="s">
+      <c r="O13" t="s">
         <v>26</v>
       </c>
-      <c r="P11" s="0" t="s">
+      <c r="P13" t="s">
         <v>27</v>
       </c>
-      <c r="Q11" s="0" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="0">
-        <v>11</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>93</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="F12" s="0">
-        <v>3</v>
-      </c>
-      <c r="G12" s="0">
-        <v>3</v>
-      </c>
-      <c r="H12" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="I12" s="0" t="s">
+      <c r="Q13" t="s">
         <v>95</v>
-      </c>
-      <c r="J12" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="K12" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="L12" s="0">
-        <v>1</v>
-      </c>
-      <c r="M12" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="N12" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="O12" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="P12" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q12" s="0" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="0">
-        <v>12</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>93</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="F13" s="0">
-        <v>3</v>
-      </c>
-      <c r="G13" s="0">
-        <v>3</v>
-      </c>
-      <c r="H13" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="I13" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="J13" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="K13" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="L13" s="0">
-        <v>1</v>
-      </c>
-      <c r="M13" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="N13" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="O13" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="P13" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q13" s="0" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Chore: Cleanup, Readme modification
</commit_message>
<xml_diff>
--- a/LaunchController1 BOM.xlsx
+++ b/LaunchController1 BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\MR-Launch-Controller\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{588297AE-1491-496B-B4A3-ED6F528889F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC876C3C-E6FA-4CAD-AFE5-206BD20C2609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="My Lists Worksheet" sheetId="1" r:id="rId1"/>
@@ -326,7 +326,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -669,13 +669,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="4" max="4" width="29.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -728,7 +728,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17">
       <c r="A2">
         <v>1</v>
       </c>
@@ -778,7 +778,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17">
       <c r="A3">
         <v>2</v>
       </c>
@@ -828,7 +828,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17">
       <c r="A4">
         <v>3</v>
       </c>
@@ -878,7 +878,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17">
       <c r="A5">
         <v>4</v>
       </c>
@@ -928,7 +928,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17">
       <c r="A6">
         <v>5</v>
       </c>
@@ -978,7 +978,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1078,7 +1078,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17">
       <c r="A13">
         <v>12</v>
       </c>

</xml_diff>